<commit_message>
adição documento de mudança
</commit_message>
<xml_diff>
--- a/HikariWasabi-Grupo6-Backlog-Burndown v2.xlsx
+++ b/HikariWasabi-Grupo6-Backlog-Burndown v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\OneDrive\Desktop\Tecnologia da informação\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{21AF9EB8-0062-47AF-B0EC-254FEB537C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E823EDCD-355E-4ABF-956A-1474B78FC908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{960F6042-E808-4157-B293-DF7D0877B487}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{960F6042-E808-4157-B293-DF7D0877B487}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -799,42 +799,11 @@
           <c:cat>
             <c:strRef>
               <c:f>Planilha1!$R$4:$R$7</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>Total</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>SP1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>SP2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>SP3</c:v>
-                </c:pt>
-              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Planilha1!$S$4:$S$7</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>393</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>170</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>123</c:v>
-                </c:pt>
-              </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -852,6 +821,7 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
+        <c:marker val="1"/>
         <c:smooth val="0"/>
         <c:axId val="797395775"/>
         <c:axId val="797393855"/>
@@ -1073,7 +1043,7 @@
             <c:strRef>
               <c:f>Planilha1!$R$15:$R$18</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Total</c:v>
                 </c:pt>
@@ -1083,9 +1053,6 @@
                 <c:pt idx="2">
                   <c:v>SP2</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>SP3</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
@@ -1094,7 +1061,7 @@
               <c:f>Planilha1!$S$15:$S$18</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>393</c:v>
                 </c:pt>
@@ -1103,9 +1070,6 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>170</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>123</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1139,7 +1103,7 @@
             <c:strRef>
               <c:f>Planilha1!$R$15:$R$18</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Total</c:v>
                 </c:pt>
@@ -1149,9 +1113,6 @@
                 <c:pt idx="2">
                   <c:v>SP2</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>SP3</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
@@ -1160,7 +1121,7 @@
               <c:f>Planilha1!$T$15:$T$18</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>393</c:v>
                 </c:pt>
@@ -1169,9 +1130,6 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>170</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>50</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2889,6 +2847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84DDDEBA-3FFC-4EB0-8A5E-4BC758C8A03B}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:T87"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2942,7 +2901,7 @@
       <c r="S2" s="18"/>
       <c r="T2" s="19"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>53</v>
       </c>
@@ -2975,7 +2934,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="27"/>
       <c r="B4" s="38"/>
       <c r="C4" s="2" t="s">
@@ -3006,7 +2965,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="27"/>
       <c r="B5" s="38" t="s">
         <v>47</v>
@@ -3039,7 +2998,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="27"/>
       <c r="B6" s="38"/>
       <c r="C6" s="2" t="s">
@@ -3070,7 +3029,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="27"/>
       <c r="B7" s="38" t="s">
         <v>9</v>
@@ -3103,7 +3062,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="27"/>
       <c r="B8" s="38"/>
       <c r="C8" s="2" t="s">
@@ -3125,7 +3084,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="27"/>
       <c r="B9" s="38"/>
       <c r="C9" s="2" t="s">
@@ -3147,7 +3106,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="27"/>
       <c r="B10" s="2" t="s">
         <v>13</v>
@@ -3171,7 +3130,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="27"/>
       <c r="B11" s="2" t="s">
         <v>8</v>
@@ -3195,7 +3154,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27"/>
       <c r="B12" s="2" t="s">
         <v>47</v>
@@ -3219,7 +3178,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="27"/>
       <c r="B13" s="2" t="s">
         <v>58</v>
@@ -3378,7 +3337,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="28" t="s">
         <v>65</v>
       </c>
@@ -3413,7 +3372,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="28"/>
       <c r="B19" s="3" t="s">
         <v>1</v>
@@ -3437,7 +3396,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="28"/>
       <c r="B20" s="3" t="s">
         <v>2</v>
@@ -3461,7 +3420,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="28"/>
       <c r="B21" s="3" t="s">
         <v>3</v>
@@ -3485,7 +3444,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="28"/>
       <c r="B22" s="3" t="s">
         <v>4</v>
@@ -3509,7 +3468,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="28"/>
       <c r="B23" s="3" t="s">
         <v>5</v>
@@ -3533,7 +3492,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="28"/>
       <c r="B24" s="3" t="s">
         <v>6</v>
@@ -3557,7 +3516,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="28"/>
       <c r="B25" s="3" t="s">
         <v>7</v>
@@ -3581,7 +3540,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="28"/>
       <c r="B26" s="3" t="s">
         <v>45</v>
@@ -3725,7 +3684,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="29" t="s">
         <v>54</v>
       </c>
@@ -3751,7 +3710,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="29"/>
       <c r="B33" s="4" t="s">
         <v>29</v>
@@ -3775,7 +3734,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="29"/>
       <c r="B34" s="4" t="s">
         <v>10</v>
@@ -3799,7 +3758,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="29"/>
       <c r="B35" s="4" t="s">
         <v>11</v>
@@ -3823,7 +3782,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="29"/>
       <c r="B36" s="4" t="s">
         <v>14</v>
@@ -4853,7 +4812,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H37" xr:uid="{84DDDEBA-3FFC-4EB0-8A5E-4BC758C8A03B}"/>
+  <autoFilter ref="A2:H37" xr:uid="{84DDDEBA-3FFC-4EB0-8A5E-4BC758C8A03B}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="SP3"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="22">
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="A47:A53"/>

</xml_diff>